<commit_message>
**Universal IFC Material Parser**
**Key features implemented:**
- Updated xlsx_parser.py to support universal material parsing beyond just concrete types
- Added detection for various materials including hydroinsulation, insulation, solutions, reinforcement using keyword mapping
- Implemented dynamic column discovery for material data in Qto_* format using regex patterns
- Enhanced material type classification with support for subtypes like membranes, mastics, primers, polystyrene
- Modified aggregation logic to handle all material categories with proper volume and count calculations
- Updated output formatting to include material type information in generated Excel reports
- Added comprehensive material column pattern matching for automatic detection of material-specific columns

The script now processes any material type from the IFC report table rather than being limited to concrete grades, providing a complete material breakdown with proper categorization and volume calculations.
</commit_message>
<xml_diff>
--- a/uploads/ad4a1618-5ed2-4986-b71d-05929dd17c31/materials_summary.xlsx
+++ b/uploads/ad4a1618-5ed2-4986-b71d-05929dd17c31/materials_summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Сводка по материалам" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка по материалам" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,13 +433,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -500,30 +500,30 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Бетон</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>марка не указана</t>
-        </is>
-      </c>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="n">
-        <v>102.775</v>
+        <v>133.605</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
+        <v>81</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>54</v>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>расчёт по объёму (8 эл.)</t>
+          <t>расчёт по объёму (81 эл.) + 54 эл. по количеству</t>
         </is>
       </c>
     </row>
@@ -533,34 +533,30 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Бетон В10</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>Бетон</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Бетон</t>
-        </is>
-      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>марка не указана</t>
+          <t>В10</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>30.83</v>
+        <v>266.561</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>54</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>расчёт по объёму (73 эл.) + 54 эл. по количеству</t>
+          <t>расчёт по объёму (8 эл.)</t>
         </is>
       </c>
     </row>
@@ -570,7 +566,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Бетон В10</t>
+          <t>Бетон В25</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -580,20 +576,20 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>В10</t>
+          <t>В25</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>266.561</v>
+        <v>2269.207</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>расчёт по объёму (8 эл.)</t>
+          <t>расчёт по объёму (66 эл.)</t>
         </is>
       </c>
     </row>
@@ -603,7 +599,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Бетон В25</t>
+          <t>Бетон В30</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -613,20 +609,20 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>В25</t>
+          <t>В30</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2269.207</v>
+        <v>3931.077</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>66</v>
+        <v>1037</v>
       </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>расчёт по объёму (66 эл.)</t>
+          <t>расчёт по объёму (1037 эл.)</t>
         </is>
       </c>
     </row>
@@ -636,7 +632,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Бетон В30</t>
+          <t>Бетон В35</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -646,51 +642,18 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>В30</t>
+          <t>В35</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>3931.077</v>
+        <v>1755.07</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1037</v>
+        <v>186</v>
       </c>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>расчёт по объёму (1037 эл.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Бетон В35</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Бетон</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>В35</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>1755.07</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>186</v>
-      </c>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>расчёт по объёму (186 эл.)</t>
         </is>

</xml_diff>

<commit_message>
Update xlsx_parser.py for universal material parsing with LLM
- Update xlsx_parser.py to use gemma4:31b LLM for intelligent material analysis, determining unit type (volume, area, length, pieces, liquid) and material group (Concrete, Waterproofing, Insulation, etc.) from material names
- Modify parsing logic to extract all material types from IFC reports, not just concrete, using LLM classification and fallback regex patterns
- Enhance data aggregation to group materials by full name, unit type, and material group, including volume (m³), area (m²), length (m), pieces (шт), and liquid volume (л)
- Update .gitignore to refine ignored file patterns and directory structure
</commit_message>
<xml_diff>
--- a/uploads/ad4a1618-5ed2-4986-b71d-05929dd17c31/materials_summary.xlsx
+++ b/uploads/ad4a1618-5ed2-4986-b71d-05929dd17c31/materials_summary.xlsx
@@ -433,10 +433,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -502,10 +502,10 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>7150.579</v>
+        <v>133.605</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>173</v>
+        <v>81</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Бетон В10</t>
+          <t>Бетон</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -525,14 +525,14 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>м³</t>
+          <t>м²</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>5545.556</v>
+        <v>7016.975</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>16</v>
+        <v>92</v>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
@@ -542,7 +542,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Бетон В25</t>
+          <t>Бетон</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -552,14 +552,14 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>м³</t>
+          <t>м</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>26240.205</v>
+        <v>601353.076</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>132</v>
+        <v>74</v>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
     </row>
@@ -569,7 +569,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Бетон В30</t>
+          <t>Бетон В10</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -583,10 +583,10 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>22102.708</v>
+        <v>266.561</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>2042</v>
+        <v>8</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Бетон В35</t>
+          <t>Бетон В10</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -606,14 +606,14 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>м³</t>
+          <t>м²</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>8578.083000000001</v>
+        <v>5278.995</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>372</v>
+        <v>8</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Бетон</t>
+          <t>Бетон В25</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -633,16 +633,232 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>м³</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>2269.207</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Бетон В25</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>23970.997</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Бетон В30</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>м³</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>3931.077</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>1037</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Бетон В30</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1283854.046</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>1037</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Бетон В30</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>м</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>3145952.806</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>1016</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Бетон В35</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>м³</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>1755.07</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>186</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Бетон В35</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>6823.014</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>186</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Бетон В35</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>м</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>640257.308</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>163</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E15" s="2" t="n">
         <v>1903</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F15" s="2" t="n">
         <v>1903</v>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Жилой дом; -1_Подземный этаж_основной; 1_Этаж_основной</t>
         </is>

</xml_diff>